<commit_message>
feat: modify excel output formatting
</commit_message>
<xml_diff>
--- a/output/five-decade-tables/usa_household_size_bedrooms_crowding_by_decade_raw.xlsx
+++ b/output/five-decade-tables/usa_household_size_bedrooms_crowding_by_decade_raw.xlsx
@@ -1,21 +1,75 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\output\five-decade-tables\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D72039D-84FA-47E2-B182-7A3FAC2DEF12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="10" yWindow="730" windowWidth="23030" windowHeight="14630" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>row</t>
+  </si>
+  <si>
+    <t>1970</t>
+  </si>
+  <si>
+    <t>1980</t>
+  </si>
+  <si>
+    <t>1990</t>
+  </si>
+  <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>2010</t>
+  </si>
+  <si>
+    <t>2020</t>
+  </si>
+  <si>
+    <t>CPS observations</t>
+  </si>
+  <si>
+    <t>ACS observations</t>
+  </si>
+  <si>
+    <t>CPS household size</t>
+  </si>
+  <si>
+    <t>ACS household size</t>
+  </si>
+  <si>
+    <t>ACS bedrooms</t>
+  </si>
+  <si>
+    <t>ACS persons per bedroom</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -31,13 +85,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,27 +122,47 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -107,7 +200,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -141,6 +234,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -175,9 +269,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -350,189 +445,178 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.42578125" customWidth="1"/>
+    <col min="2" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>row</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>1970</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>1980</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>1990</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CPS observations</t>
-        </is>
-      </c>
-      <c r="B2">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="9">
         <v>145023</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="9">
         <v>181488</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="9">
         <v>158079</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="9">
         <v>133710</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="9">
         <v>209802</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="9">
         <v>157959</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ACS observations</t>
-        </is>
-      </c>
-      <c r="B3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="11">
         <v>1972044</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="11">
         <v>2209919</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="11">
         <v>2447860</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="11">
         <v>2740185</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="11">
         <v>30065222</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="11">
         <v>14884820</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CPS household size</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>4.225605469731446</v>
-      </c>
-      <c r="C4">
-        <v>3.625101641700611</v>
-      </c>
-      <c r="D4">
-        <v>3.420819395241213</v>
-      </c>
-      <c r="E4">
-        <v>3.402339305668489</v>
-      </c>
-      <c r="F4">
-        <v>3.394128895563963</v>
-      </c>
-      <c r="G4">
-        <v>3.311556108369965</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ACS household size</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>4.173105671070219</v>
-      </c>
-      <c r="C5">
-        <v>3.628820332328922</v>
-      </c>
-      <c r="D5">
-        <v>3.47123949474108</v>
-      </c>
-      <c r="E5">
-        <v>3.469581955413218</v>
-      </c>
-      <c r="F5">
-        <v>3.493749222939381</v>
-      </c>
-      <c r="G5">
-        <v>3.361668366067391</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ACS bedrooms</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>2.750220583313557</v>
-      </c>
-      <c r="C6">
-        <v>2.793488358623099</v>
-      </c>
-      <c r="D6">
-        <v>2.811066824944201</v>
-      </c>
-      <c r="E6">
+    <row r="4" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3">
+        <v>4.2256054697314456</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.6251016417006112</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3.4208193952412129</v>
+      </c>
+      <c r="E5" s="3">
+        <v>3.4023393056684892</v>
+      </c>
+      <c r="F5" s="3">
+        <v>3.3941288955639628</v>
+      </c>
+      <c r="G5" s="3">
+        <v>3.3115561083699649</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="5">
+        <v>4.1731056710702186</v>
+      </c>
+      <c r="C6" s="5">
+        <v>3.6288203323289219</v>
+      </c>
+      <c r="D6" s="5">
+        <v>3.4712394947410798</v>
+      </c>
+      <c r="E6" s="5">
+        <v>3.4695819554132181</v>
+      </c>
+      <c r="F6" s="5">
+        <v>3.4937492229393809</v>
+      </c>
+      <c r="G6" s="5">
+        <v>3.3616683660673909</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="5">
+        <v>2.7502205833135571</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2.7934883586230992</v>
+      </c>
+      <c r="D7" s="5">
+        <v>2.8110668249442008</v>
+      </c>
+      <c r="E7" s="5">
         <v>2.823591041819685</v>
       </c>
-      <c r="G6">
-        <v>3.028105463751085</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ACS persons per bedroom</t>
-        </is>
-      </c>
-      <c r="B7">
+      <c r="F7" s="5"/>
+      <c r="G7" s="5">
+        <v>3.0281054637510851</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="5">
         <v>1.605259272443563</v>
       </c>
-      <c r="C7">
+      <c r="C8" s="5">
         <v>1.385040605560643</v>
       </c>
-      <c r="D7">
+      <c r="D8" s="5">
         <v>1.365724182779857</v>
       </c>
-      <c r="E7">
+      <c r="E8" s="5">
         <v>1.397949369188221</v>
       </c>
-      <c r="G7">
-        <v>1.188879882358216</v>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5">
+        <v>1.1888798823582161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: make more summary graphs
</commit_message>
<xml_diff>
--- a/output/five-decade-tables/usa_household_size_bedrooms_crowding_by_decade_raw.xlsx
+++ b/output/five-decade-tables/usa_household_size_bedrooms_crowding_by_decade_raw.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\output\five-decade-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15DFB830-2EA8-4FF6-939D-5F120E6439AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A75E52-BDD3-4BBB-B71D-0D4E2A6280A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="730" windowWidth="23030" windowHeight="14630" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -67,7 +80,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -133,8 +146,8 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -154,6 +167,910 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ACS bedrooms</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$1:$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1970</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1980</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1990</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2010</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2020</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$7:$G$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2.7502205833135571</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.7934883586230992</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8110668249442008</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.823591041819685</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.9922654899110959</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.0281054637510851</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-647C-4057-B3F5-ABAECD986F0A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1846441072"/>
+        <c:axId val="1846441552"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1846441072"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1846441552"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1846441552"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1846441072"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>873125</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75DF477D-3D9A-8E0D-DFCB-11BCF2F4B10D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -444,14 +1361,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.7265625" customWidth="1"/>
+    <col min="2" max="5" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,7 +1391,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
@@ -497,7 +1414,7 @@
         <v>157959</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
@@ -520,10 +1437,10 @@
         <v>14884820</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="8"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
@@ -546,7 +1463,7 @@
         <v>3.3115561083699649</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
@@ -569,7 +1486,7 @@
         <v>3.3616683660673909</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>11</v>
       </c>
@@ -592,7 +1509,7 @@
         <v>3.0281054637510851</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>12</v>
       </c>
@@ -617,5 +1534,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>